<commit_message>
[vikas] newly written transactions And it's IO files, Updated APIs validation classes along with deleted unwanted files
</commit_message>
<xml_diff>
--- a/src/main/resources/menuItems/purchase/transactions/461617 - Purchase Enquiries-AC_PE_3_Output.xlsx
+++ b/src/main/resources/menuItems/purchase/transactions/461617 - Purchase Enquiries-AC_PE_3_Output.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\IdeaProjects\wings-testautomation\src\main\resources\menuItems\purchase\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8FB53FB-0226-41F1-A3F3-E68E76462B1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F000BDD-7CF0-4BFF-8502-DE3B0E9623EC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="952"/>
+    <workbookView xWindow="32760" yWindow="32760" windowWidth="32760" windowHeight="32760" tabRatio="952" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="358">
   <si>
     <t>TableNames</t>
   </si>
@@ -337,9 +337,6 @@
     <t>24D Books Fin AT</t>
   </si>
   <si>
-    <t>PVREM1</t>
-  </si>
-  <si>
     <t>ProductCode</t>
   </si>
   <si>
@@ -623,21 +620,6 @@
   </si>
   <si>
     <t>PVRBN11</t>
-  </si>
-  <si>
-    <t>PVOI1</t>
-  </si>
-  <si>
-    <t>PVOI3</t>
-  </si>
-  <si>
-    <t>PVOI4</t>
-  </si>
-  <si>
-    <t>PVOI5</t>
-  </si>
-  <si>
-    <t>PVOI2</t>
   </si>
   <si>
     <t>PVAI1</t>
@@ -1156,7 +1138,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1503,7 +1485,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -1961,7 +1943,51 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.69999998807907104" right="0.69999998807907104" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
+  <pageSetup errors="blank"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2004,8 +2030,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2048,8 +2074,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2092,52 +2118,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr autoPageBreaks="0"/>
-  </sheetPr>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.69999998807907104" right="0.69999998807907104" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
-  <pageSetup errors="blank"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2146,22 +2128,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="B1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" t="s">
         <v>113</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>114</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>115</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>116</v>
-      </c>
-      <c r="F1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2271,7 +2253,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2283,32 +2265,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2318,7 +2300,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2330,32 +2312,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2365,7 +2347,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2412,7 +2394,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2424,7 +2406,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2439,7 +2421,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2486,7 +2468,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2498,7 +2480,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2508,7 +2490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2527,7 +2509,7 @@
         <v>69</v>
       </c>
       <c r="B1" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="C1" t="s">
         <v>68</v>
@@ -2536,7 +2518,7 @@
         <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -2553,7 +2535,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -2563,7 +2545,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1400-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2572,16 +2554,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
         <v>121</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>122</v>
       </c>
-      <c r="C1" t="s">
-        <v>123</v>
-      </c>
       <c r="D1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2605,7 +2587,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1500-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2618,16 +2600,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" t="s">
         <v>118</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>119</v>
       </c>
-      <c r="C1" t="s">
-        <v>120</v>
-      </c>
       <c r="D1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2651,7 +2633,31 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1600-000000000000}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.69999998807907104" right="0.69999998807907104" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
+  <pageSetup errors="blank"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1700-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2665,7 +2671,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2674,8 +2680,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1800-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2689,7 +2695,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2698,8 +2704,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1900-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2713,7 +2719,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2722,8 +2728,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1A00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2737,31 +2743,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.69999998807907104" right="0.69999998807907104" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
-  <pageSetup errors="blank"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr autoPageBreaks="0"/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2771,7 +2753,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2780,22 +2762,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="B1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" t="s">
         <v>113</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>114</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>115</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>116</v>
-      </c>
-      <c r="F1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -2825,7 +2807,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1C00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2852,7 +2834,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -2869,25 +2851,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="C1" t="s">
         <v>75</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2901,16 +2883,13 @@
         <v>88</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E2">
-        <v>1.123</v>
+        <v>123</v>
       </c>
       <c r="F2">
         <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2924,16 +2903,13 @@
         <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E3">
-        <v>1.1240000000000001</v>
+        <v>135</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -2947,16 +2923,13 @@
         <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4">
-        <v>1.1259999999999999</v>
+        <v>146</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -2970,7 +2943,7 @@
         <v>88</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -2979,7 +2952,7 @@
         <v>250</v>
       </c>
       <c r="G5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -2993,7 +2966,7 @@
         <v>88</v>
       </c>
       <c r="D6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E6">
         <v>1.1200000000000001</v>
@@ -3002,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3012,7 +2985,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1D00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3039,7 +3012,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1E00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3051,57 +3024,57 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -3111,11 +3084,11 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1F00-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -3123,36 +3096,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B1" t="s">
         <v>182</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>183</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>184</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>185</v>
-      </c>
-      <c r="E1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E2" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3162,7 +3118,7 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2000-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3174,32 +3130,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3209,7 +3165,7 @@
 </file>
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2100-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3221,32 +3177,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -3256,7 +3212,7 @@
 </file>
 
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2200-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3272,19 +3228,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="B1" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="C1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E1" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -3298,10 +3254,10 @@
         <v>45895</v>
       </c>
       <c r="D2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>
@@ -3311,21 +3267,16 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2300-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -3335,7 +3286,7 @@
 </file>
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2400-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3351,19 +3302,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
         <v>77</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -3373,7 +3324,7 @@
 </file>
 
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2500-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3386,50 +3337,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B2" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B6" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3439,7 +3390,7 @@
 </file>
 
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2600-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3466,7 +3417,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3489,22 +3440,22 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B1" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C1" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D1" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="E1" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="F1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="G1" t="s">
         <v>71</v>
@@ -3513,16 +3464,16 @@
         <v>74</v>
       </c>
       <c r="I1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L1" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -3551,10 +3502,10 @@
         <v>87</v>
       </c>
       <c r="I2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J2" t="s">
         <v>124</v>
-      </c>
-      <c r="J2" t="s">
-        <v>125</v>
       </c>
       <c r="K2">
         <v>100</v>
@@ -3589,10 +3540,10 @@
         <v>87</v>
       </c>
       <c r="I3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -3627,10 +3578,10 @@
         <v>87</v>
       </c>
       <c r="I4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="J4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -3665,10 +3616,10 @@
         <v>87</v>
       </c>
       <c r="I5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K5">
         <v>250</v>
@@ -3703,10 +3654,10 @@
         <v>87</v>
       </c>
       <c r="I6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -3722,7 +3673,7 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-2700-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3749,7 +3700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -3834,76 +3785,76 @@
   <sheetData>
     <row r="1" spans="1:81" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B1" t="s">
         <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="E1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="F1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="G1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="H1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J1" t="s">
         <v>68</v>
       </c>
       <c r="K1" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" t="s">
+        <v>102</v>
+      </c>
+      <c r="M1" t="s">
+        <v>223</v>
+      </c>
+      <c r="N1" t="s">
+        <v>224</v>
+      </c>
+      <c r="O1" t="s">
+        <v>225</v>
+      </c>
+      <c r="P1" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>227</v>
+      </c>
+      <c r="R1" t="s">
         <v>228</v>
-      </c>
-      <c r="L1" t="s">
-        <v>103</v>
-      </c>
-      <c r="M1" t="s">
-        <v>229</v>
-      </c>
-      <c r="N1" t="s">
-        <v>230</v>
-      </c>
-      <c r="O1" t="s">
-        <v>231</v>
-      </c>
-      <c r="P1" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>233</v>
-      </c>
-      <c r="R1" t="s">
-        <v>234</v>
       </c>
       <c r="S1" t="s">
         <v>77</v>
       </c>
       <c r="T1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="U1" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="V1" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="W1" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="X1" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="Y1" t="s">
         <v>66</v>
@@ -3912,169 +3863,169 @@
         <v>76</v>
       </c>
       <c r="AA1" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>235</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>237</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>238</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>239</v>
+      </c>
+      <c r="AH1" t="s">
         <v>240</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AI1" t="s">
         <v>241</v>
       </c>
-      <c r="AC1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AD1" t="s">
+      <c r="AJ1" t="s">
         <v>242</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AK1" t="s">
         <v>243</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AL1" t="s">
         <v>244</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AM1" t="s">
         <v>245</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AN1" t="s">
+        <v>94</v>
+      </c>
+      <c r="AO1" t="s">
         <v>246</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AP1" t="s">
         <v>247</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AQ1" t="s">
         <v>248</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AR1" t="s">
         <v>249</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>250</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>251</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>95</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>252</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>253</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>254</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>255</v>
       </c>
       <c r="AS1" t="s">
         <v>74</v>
       </c>
       <c r="AT1" t="s">
+        <v>250</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>251</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>92</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>98</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>99</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>252</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>253</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>254</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>255</v>
+      </c>
+      <c r="BF1" t="s">
         <v>256</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BG1" t="s">
         <v>257</v>
       </c>
-      <c r="AV1" t="s">
-        <v>94</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>99</v>
-      </c>
-      <c r="BA1" t="s">
+      <c r="BH1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>258</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>259</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>260</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>261</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>262</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>263</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>264</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>265</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>266</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>268</v>
+      </c>
+      <c r="BT1" t="s">
         <v>100</v>
       </c>
-      <c r="BB1" t="s">
-        <v>258</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>259</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>260</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>261</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>262</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BH1" t="s">
+      <c r="BU1" t="s">
         <v>96</v>
       </c>
-      <c r="BI1" t="s">
-        <v>264</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>265</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>266</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>267</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>268</v>
-      </c>
-      <c r="BN1" t="s">
+      <c r="BV1" t="s">
         <v>269</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BW1" t="s">
         <v>270</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BX1" t="s">
         <v>271</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BY1" t="s">
         <v>272</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BZ1" t="s">
         <v>273</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CA1" t="s">
         <v>274</v>
       </c>
-      <c r="BT1" t="s">
-        <v>101</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>97</v>
-      </c>
-      <c r="BV1" t="s">
+      <c r="CB1" t="s">
         <v>275</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CC1" t="s">
         <v>276</v>
-      </c>
-      <c r="BX1" t="s">
-        <v>277</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>278</v>
-      </c>
-      <c r="BZ1" t="s">
-        <v>279</v>
-      </c>
-      <c r="CA1" t="s">
-        <v>280</v>
-      </c>
-      <c r="CB1" t="s">
-        <v>281</v>
-      </c>
-      <c r="CC1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:81" x14ac:dyDescent="0.25">
@@ -4103,7 +4054,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J2" s="1">
         <v>45849</v>
@@ -4112,7 +4063,7 @@
         <v>45866.638870158502</v>
       </c>
       <c r="L2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -4184,7 +4135,7 @@
         <v>88</v>
       </c>
       <c r="AJ2" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AK2">
         <v>0</v>
@@ -4220,16 +4171,16 @@
         <v>0</v>
       </c>
       <c r="AV2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AW2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AX2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AY2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AZ2">
         <v>1.123</v>
@@ -4256,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="BH2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BI2">
         <v>0</v>
@@ -4295,7 +4246,7 @@
         <v>100</v>
       </c>
       <c r="BU2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BV2">
         <v>0</v>
@@ -4348,7 +4299,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J3" s="1">
         <v>45849</v>
@@ -4357,7 +4308,7 @@
         <v>45866.638870379044</v>
       </c>
       <c r="L3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -4429,7 +4380,7 @@
         <v>88</v>
       </c>
       <c r="AJ3" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AK3">
         <v>0</v>
@@ -4465,16 +4416,16 @@
         <v>0</v>
       </c>
       <c r="AV3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AX3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AY3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AZ3">
         <v>1.1240000000000001</v>
@@ -4501,7 +4452,7 @@
         <v>0</v>
       </c>
       <c r="BH3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BI3">
         <v>0</v>
@@ -4540,7 +4491,7 @@
         <v>0</v>
       </c>
       <c r="BU3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BV3">
         <v>0</v>
@@ -4593,7 +4544,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J4" s="1">
         <v>45849</v>
@@ -4602,7 +4553,7 @@
         <v>45866.638870425573</v>
       </c>
       <c r="L4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="M4">
         <v>0</v>
@@ -4674,7 +4625,7 @@
         <v>88</v>
       </c>
       <c r="AJ4" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AK4">
         <v>0</v>
@@ -4710,16 +4661,16 @@
         <v>0</v>
       </c>
       <c r="AV4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AW4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AX4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AY4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AZ4">
         <v>1.1259999999999999</v>
@@ -4746,7 +4697,7 @@
         <v>0</v>
       </c>
       <c r="BH4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BI4">
         <v>0</v>
@@ -4785,7 +4736,7 @@
         <v>0</v>
       </c>
       <c r="BU4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BV4">
         <v>0</v>
@@ -4838,7 +4789,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J5" s="1">
         <v>45849</v>
@@ -4847,7 +4798,7 @@
         <v>45866.638870465278</v>
       </c>
       <c r="L5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -4919,7 +4870,7 @@
         <v>88</v>
       </c>
       <c r="AJ5" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AK5">
         <v>0</v>
@@ -4955,16 +4906,16 @@
         <v>0</v>
       </c>
       <c r="AV5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AW5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AX5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AY5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AZ5">
         <v>1</v>
@@ -4991,7 +4942,7 @@
         <v>0</v>
       </c>
       <c r="BH5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BI5">
         <v>0</v>
@@ -5030,7 +4981,7 @@
         <v>250</v>
       </c>
       <c r="BU5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BV5">
         <v>0</v>
@@ -5083,7 +5034,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J6" s="1">
         <v>45849</v>
@@ -5092,7 +5043,7 @@
         <v>45866.638870504925</v>
       </c>
       <c r="L6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="M6">
         <v>0</v>
@@ -5164,7 +5115,7 @@
         <v>88</v>
       </c>
       <c r="AJ6" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AK6">
         <v>0</v>
@@ -5200,16 +5151,16 @@
         <v>0</v>
       </c>
       <c r="AV6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AW6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AX6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AY6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AZ6">
         <v>1.1200000000000001</v>
@@ -5236,7 +5187,7 @@
         <v>0</v>
       </c>
       <c r="BH6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BI6">
         <v>0</v>
@@ -5275,7 +5226,7 @@
         <v>0</v>
       </c>
       <c r="BU6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="BV6">
         <v>0</v>
@@ -5309,7 +5260,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -5416,61 +5367,61 @@
   <sheetData>
     <row r="1" spans="1:101" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="B1" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="C1" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="D1" t="s">
         <v>69</v>
       </c>
       <c r="E1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="F1" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="G1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="H1" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="I1" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="J1" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="K1" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="L1" t="s">
         <v>68</v>
       </c>
       <c r="M1" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="N1" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="O1" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="P1" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="Q1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="R1" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="S1" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="T1" t="s">
         <v>66</v>
@@ -5479,100 +5430,100 @@
         <v>72</v>
       </c>
       <c r="V1" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="W1" t="s">
         <v>76</v>
       </c>
       <c r="X1" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="Y1" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="Z1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA1" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="AB1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="AC1" t="s">
+        <v>293</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>294</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>295</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>296</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>297</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>298</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>243</v>
+      </c>
+      <c r="AJ1" t="s">
         <v>299</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AK1" t="s">
         <v>300</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AL1" t="s">
         <v>301</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AM1" t="s">
         <v>302</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AN1" t="s">
         <v>303</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AO1" t="s">
         <v>304</v>
       </c>
-      <c r="AI1" t="s">
-        <v>249</v>
-      </c>
-      <c r="AJ1" t="s">
+      <c r="AP1" t="s">
         <v>305</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AQ1" t="s">
+        <v>247</v>
+      </c>
+      <c r="AR1" t="s">
         <v>306</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AS1" t="s">
         <v>307</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AT1" t="s">
         <v>308</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AU1" t="s">
         <v>309</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AV1" t="s">
         <v>310</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AW1" t="s">
         <v>311</v>
       </c>
-      <c r="AQ1" t="s">
-        <v>253</v>
-      </c>
-      <c r="AR1" t="s">
+      <c r="AX1" t="s">
         <v>312</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AY1" t="s">
         <v>313</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AZ1" t="s">
         <v>314</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="BA1" t="s">
         <v>315</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>316</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>317</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>318</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>319</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>320</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>321</v>
       </c>
       <c r="BB1" t="s">
         <v>74</v>
@@ -5581,142 +5532,142 @@
         <v>73</v>
       </c>
       <c r="BD1" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="BE1" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="BF1" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="BG1" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="BH1" t="s">
         <v>75</v>
       </c>
       <c r="BI1" t="s">
+        <v>98</v>
+      </c>
+      <c r="BJ1" t="s">
         <v>99</v>
       </c>
-      <c r="BJ1" t="s">
-        <v>100</v>
-      </c>
       <c r="BK1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BL1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="BM1" t="s">
+        <v>320</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>321</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>322</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>323</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>256</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>324</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>325</v>
+      </c>
+      <c r="BT1" t="s">
         <v>326</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BU1" t="s">
+        <v>258</v>
+      </c>
+      <c r="BV1" t="s">
         <v>327</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BW1" t="s">
         <v>328</v>
       </c>
-      <c r="BP1" t="s">
+      <c r="BX1" t="s">
         <v>329</v>
       </c>
-      <c r="BQ1" t="s">
-        <v>262</v>
-      </c>
-      <c r="BR1" t="s">
+      <c r="BY1" t="s">
         <v>330</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="BZ1" t="s">
         <v>331</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CA1" t="s">
         <v>332</v>
       </c>
-      <c r="BU1" t="s">
-        <v>264</v>
-      </c>
-      <c r="BV1" t="s">
+      <c r="CB1" t="s">
         <v>333</v>
       </c>
-      <c r="BW1" t="s">
+      <c r="CC1" t="s">
         <v>334</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CD1" t="s">
         <v>335</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CE1" t="s">
         <v>336</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CF1" t="s">
         <v>337</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CG1" t="s">
         <v>338</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CH1" t="s">
         <v>339</v>
-      </c>
-      <c r="CC1" t="s">
-        <v>340</v>
-      </c>
-      <c r="CD1" t="s">
-        <v>341</v>
-      </c>
-      <c r="CE1" t="s">
-        <v>342</v>
-      </c>
-      <c r="CF1" t="s">
-        <v>343</v>
-      </c>
-      <c r="CG1" t="s">
-        <v>344</v>
-      </c>
-      <c r="CH1" t="s">
-        <v>345</v>
       </c>
       <c r="CI1" t="s">
         <v>70</v>
       </c>
       <c r="CJ1" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="CK1" t="s">
+        <v>340</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>341</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>342</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>343</v>
+      </c>
+      <c r="CO1" t="s">
+        <v>344</v>
+      </c>
+      <c r="CP1" t="s">
+        <v>345</v>
+      </c>
+      <c r="CQ1" t="s">
         <v>346</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="CR1" t="s">
         <v>347</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="CS1" t="s">
         <v>348</v>
       </c>
-      <c r="CN1" t="s">
-        <v>349</v>
-      </c>
-      <c r="CO1" t="s">
-        <v>350</v>
-      </c>
-      <c r="CP1" t="s">
-        <v>351</v>
-      </c>
-      <c r="CQ1" t="s">
-        <v>352</v>
-      </c>
-      <c r="CR1" t="s">
-        <v>353</v>
-      </c>
-      <c r="CS1" t="s">
-        <v>354</v>
-      </c>
       <c r="CT1" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="CU1" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="CV1" t="s">
         <v>67</v>
       </c>
       <c r="CW1" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" spans="1:101" x14ac:dyDescent="0.25">
@@ -5817,7 +5768,7 @@
         <v>86</v>
       </c>
       <c r="AG2" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="AH2" t="s">
         <v>88</v>
@@ -5889,13 +5840,13 @@
         <v>88</v>
       </c>
       <c r="BE2" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="BF2" t="s">
         <v>88</v>
       </c>
       <c r="BG2" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="BH2" t="s">
         <v>89</v>
@@ -5910,7 +5861,7 @@
         <v>45895</v>
       </c>
       <c r="BL2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BM2">
         <v>0</v>
@@ -5943,7 +5894,7 @@
         <v>88</v>
       </c>
       <c r="BW2" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="BX2">
         <v>0</v>
@@ -6000,7 +5951,7 @@
         <v>88</v>
       </c>
       <c r="CP2" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="CQ2">
         <v>0</v>
@@ -6031,7 +5982,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -6044,16 +5995,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
         <v>121</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>122</v>
       </c>
-      <c r="C1" t="s">
-        <v>123</v>
-      </c>
       <c r="D1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -6133,7 +6084,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -6146,16 +6097,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B1" t="s">
         <v>118</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>119</v>
       </c>
-      <c r="C1" t="s">
-        <v>120</v>
-      </c>
       <c r="D1" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -6235,7 +6186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
@@ -6244,32 +6195,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>